<commit_message>
Phase 3: Start and Bedrijf & Contact sheets
Start sheet: welcome text, consultant contact block, 6-item
attachments checklist with ☐/☑ dropdown, progress counter
(COUNTA of required refs / total), comments block.
Bedrijf & Contact sheet: company NAW, HR contact, Finance
contact, bank details (IBAN required, BIC optional for
non-SEPA). Cell comments added for non-trivial fields.
11 required fields registered, 0 formula errors, 17.3 KB.

https://claude.ai/code/session_01QG7xshNkELyspBZLGsyRFs
</commit_message>
<xml_diff>
--- a/outputs/Payroll_Discovery_Document_MKB.xlsx
+++ b/outputs/Payroll_Discovery_Document_MKB.xlsx
@@ -39,7 +39,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -56,8 +56,41 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="007F7F7F"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F3864"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00595959"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00C00000"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -69,8 +102,23 @@
         <fgColor rgb="001F3864"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E1F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -78,14 +126,61 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -162,6 +257,66 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>SD Worx</author>
+  </authors>
+  <commentList>
+    <comment ref="B8" authorId="0" shapeId="0">
+      <text>
+        <t>In te vullen door SD Worx-consultant.</t>
+      </text>
+    </comment>
+    <comment ref="B9" authorId="0" shapeId="0">
+      <text>
+        <t>In te vullen door SD Worx-consultant.</t>
+      </text>
+    </comment>
+    <comment ref="B10" authorId="0" shapeId="0">
+      <text>
+        <t>In te vullen door SD Worx-consultant.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>SD Worx</author>
+  </authors>
+  <commentList>
+    <comment ref="B6" authorId="0" shapeId="0">
+      <text>
+        <t>Formaat: 1234 AB</t>
+      </text>
+    </comment>
+    <comment ref="B8" authorId="0" shapeId="0">
+      <text>
+        <t>8 cijfers, zonder vestigingsnummer.</t>
+      </text>
+    </comment>
+    <comment ref="B9" authorId="0" shapeId="0">
+      <text>
+        <t>Formaat: 123456789L01. Wordt ook gevraagd op tab 3. Loonheffing; hier mag u overslaan.</t>
+      </text>
+    </comment>
+    <comment ref="B24" authorId="0" shapeId="0">
+      <text>
+        <t>Nederlands IBAN, bijv. NL91 ABNA 0417 1643 00. Spaties mogen, worden genegeerd.</t>
+      </text>
+    </comment>
+    <comment ref="B26" authorId="0" shapeId="0">
+      <text>
+        <t>Alleen invullen als de bank NIET in de IBAN-zone (Europa) zit.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -453,7 +608,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -473,14 +628,212 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Welkom! Dit document is de basis voor de inrichting van uw loonadministratie in Cobra (SD Worx).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Vul per tabblad de gegevens in. Geschatte invultijd: 30 - 45 minuten. Velden met * zijn verplicht.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Geel = door u in te vullen.   Lichtgrijs = voorstel (overschrijfbaar).   Bij twijfel: leeglaten en contact opnemen met uw consultant.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Uw contactpersoon bij SD Worx</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Naam consultant</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>E-mail</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>Telefoon</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="n"/>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Benodigde bijlagen  (aanvinken wat is meegestuurd)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>Kopie laatste loonstrook van ca. 5 medewerkers (incl. 1 met variabele beloning, 1 met pensioen)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>Kopie WHK-beschikking lopend jaar</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>Kopie grootboekschema + laatste journaalpost (alleen als u GL-export wilt)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>Kopie pensioenregeling (alleen als u NIET bij een bedrijfstakpensioenfonds zit)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>CAO (alleen als van toepassing)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>Functielijst (functiecode + omschrijving)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Voortgang verplichte velden</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>Aantal ingevuld / totaal</t>
+        </is>
+      </c>
+      <c r="B21" s="10">
+        <f>COUNTA('1. Bedrijf &amp; Contact'!$B$4,'1. Bedrijf &amp; Contact'!$B$5,'1. Bedrijf &amp; Contact'!$B$6,'1. Bedrijf &amp; Contact'!$B$7,'1. Bedrijf &amp; Contact'!$B$12,'1. Bedrijf &amp; Contact'!$B$14,'1. Bedrijf &amp; Contact'!$B$15,'1. Bedrijf &amp; Contact'!$B$18,'1. Bedrijf &amp; Contact'!$B$20,'1. Bedrijf &amp; Contact'!$B$21,'1. Bedrijf &amp; Contact'!$B$24)&amp;" / 11"</f>
+        <v/>
+      </c>
+      <c r="C21" s="11" t="inlineStr">
+        <is>
+          <t>Tip: sla het bestand op of druk op F9 om de teller te verversen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>Percentage ingevuld</t>
+        </is>
+      </c>
+      <c r="B22" s="10">
+        <f>IFERROR(TEXT(COUNTA('1. Bedrijf &amp; Contact'!$B$4,'1. Bedrijf &amp; Contact'!$B$5,'1. Bedrijf &amp; Contact'!$B$6,'1. Bedrijf &amp; Contact'!$B$7,'1. Bedrijf &amp; Contact'!$B$12,'1. Bedrijf &amp; Contact'!$B$14,'1. Bedrijf &amp; Contact'!$B$15,'1. Bedrijf &amp; Contact'!$B$18,'1. Bedrijf &amp; Contact'!$B$20,'1. Bedrijf &amp; Contact'!$B$21,'1. Bedrijf &amp; Contact'!$B$24)/11,"0%"),"0%")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Opmerkingen</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="12" t="n"/>
+    </row>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
-  <mergeCells count="1">
+  <mergeCells count="15">
     <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A4:H4"/>
+    <mergeCell ref="A12:H12"/>
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="B14:H14"/>
+    <mergeCell ref="B17:H17"/>
+    <mergeCell ref="B18:H18"/>
+    <mergeCell ref="A7:H7"/>
+    <mergeCell ref="B13:H13"/>
+    <mergeCell ref="A20:H20"/>
+    <mergeCell ref="A24:H24"/>
+    <mergeCell ref="A25:H28"/>
+    <mergeCell ref="B16:H16"/>
+    <mergeCell ref="B15:H15"/>
+    <mergeCell ref="A5:H5"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="A13 A14 A15 A16 A17 A18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ongeldige invoer" error="Ongeldige keuze. Kies uit de lijst." type="list">
+      <formula1>=val_Checkbox</formula1>
+    </dataValidation>
+  </dataValidations>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -490,7 +843,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -510,14 +863,205 @@
         </is>
       </c>
     </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Bedrijfsgegevens</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="13" t="inlineStr">
+        <is>
+          <t>Bedrijfsnaam *</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>Straat + huisnummer *</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="13" t="inlineStr">
+        <is>
+          <t>Postcode *</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="13" t="inlineStr">
+        <is>
+          <t>Plaats *</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>KvK-nummer</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>Loonheffingsnummer</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="n"/>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Contactpersoon HR / salarisadministratie</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="13" t="inlineStr">
+        <is>
+          <t>Naam *</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>Functie</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="13" t="inlineStr">
+        <is>
+          <t>Telefoon *</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="13" t="inlineStr">
+        <is>
+          <t>E-mail *</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="n"/>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Contactpersoon Finance / boekhouding</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="13" t="inlineStr">
+        <is>
+          <t>Naam *</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>Functie</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="13" t="inlineStr">
+        <is>
+          <t>Telefoon *</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="13" t="inlineStr">
+        <is>
+          <t>E-mail *</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="n"/>
+    </row>
+    <row r="23" ht="22" customHeight="1">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>Bankgegevens (voor SEPA-betaalbestand nettolonen)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="13" t="inlineStr">
+        <is>
+          <t>IBAN-rekeningnummer *</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>Naam bank</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>BIC / SWIFT-code</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>* = verplicht veld. Niet-verplichte velden mogen leeg blijven.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="22" customHeight="1">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Opmerkingen</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="12" t="n"/>
+    </row>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
-  <mergeCells count="1">
+  <mergeCells count="7">
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A30:H30"/>
+    <mergeCell ref="A31:H34"/>
+    <mergeCell ref="A11:H11"/>
     <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A23:H23"/>
+    <mergeCell ref="A17:H17"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -732,72 +1276,72 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="14" t="inlineStr">
         <is>
           <t>val_JaNee</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="14" t="inlineStr">
         <is>
           <t>val_Salarisperiode</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="14" t="inlineStr">
         <is>
           <t>val_Taal</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="14" t="inlineStr">
         <is>
           <t>val_Indeling</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="14" t="inlineStr">
         <is>
           <t>val_Oproep</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="14" t="inlineStr">
         <is>
           <t>val_Maand</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G1" s="14" t="inlineStr">
         <is>
           <t>val_Zichtbaarheid</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H1" s="14" t="inlineStr">
         <is>
           <t>val_Formaat</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="I1" s="14" t="inlineStr">
         <is>
           <t>val_Basisperiode</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="J1" s="14" t="inlineStr">
         <is>
           <t>val_FinSysteem</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="K1" s="14" t="inlineStr">
         <is>
           <t>val_30pct</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="L1" s="14" t="inlineStr">
         <is>
           <t>val_Toggle</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="M1" s="14" t="inlineStr">
         <is>
           <t>val_Checkbox</t>
         </is>
       </c>
-      <c r="N1" s="2" t="inlineStr">
+      <c r="N1" s="14" t="inlineStr">
         <is>
           <t>val_Sector</t>
         </is>

</xml_diff>

<commit_message>
Phase 4: Payroll basis and Loonheffing sheets
Payroll basis: CAO yes/no + name, hours/week (default 40),
hours/day mon-fri (defaults 8), wage period (default Maand),
payslip language/logo/visibility, 30% ruling (3 options), trainee
and on-call employee types.
Loonheffing: tax number, sector (67-item dropdown), employer
classification, CBS code, WBSO. WHK shown as attachment-only
info block (no premium fields).
24 required fields total, 0 formula errors, 22.2 KB.

https://claude.ai/code/session_01QG7xshNkELyspBZLGsyRFs
</commit_message>
<xml_diff>
--- a/outputs/Payroll_Discovery_Document_MKB.xlsx
+++ b/outputs/Payroll_Discovery_Document_MKB.xlsx
@@ -90,7 +90,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -115,6 +115,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF8E7"/>
       </patternFill>
     </fill>
   </fills>
@@ -144,7 +149,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -181,6 +186,16 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -313,6 +328,91 @@
     <comment ref="B26" authorId="0" shapeId="0">
       <text>
         <t>Alleen invullen als de bank NIET in de IBAN-zone (Europa) zit.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment3.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>SD Worx</author>
+  </authors>
+  <commentList>
+    <comment ref="B5" authorId="0" shapeId="0">
+      <text>
+        <t>Voluit de officiele naam, bv. 'CAO Metaal en Techniek'.</t>
+      </text>
+    </comment>
+    <comment ref="B8" authorId="0" shapeId="0">
+      <text>
+        <t>Standaard fulltime = 40 uur. Wijk alleen af als uw CAO iets anders voorschrijft.</t>
+      </text>
+    </comment>
+    <comment ref="B12" authorId="0" shapeId="0">
+      <text>
+        <t>Voor MKB bijna altijd 'Maand'. '4 weken' enkel bij CAO-verplichting.</t>
+      </text>
+    </comment>
+    <comment ref="B16" authorId="0" shapeId="0">
+      <text>
+        <t>Bij 'Ja': stuur het logo als PNG of JPG mee (min. 300 dpi).</t>
+      </text>
+    </comment>
+    <comment ref="B18" authorId="0" shapeId="0">
+      <text>
+        <t>Alleen invullen als hierboven '# dagen na de betaaldatum' is gekozen.</t>
+      </text>
+    </comment>
+    <comment ref="B21" authorId="0" shapeId="0">
+      <text>
+        <t>Kies 'Nee' als u geen buitenlandse kenniswerkers in dienst heeft.</t>
+      </text>
+    </comment>
+    <comment ref="B22" authorId="0" shapeId="0">
+      <text>
+        <t>Alleen invullen bij 'Ja' hierboven.</t>
+      </text>
+    </comment>
+    <comment ref="B26" authorId="0" shapeId="0">
+      <text>
+        <t>Kies het type oproepovereenkomst. Bij meerdere soorten: kies 'Ja, beide'.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment4.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>SD Worx</author>
+  </authors>
+  <commentList>
+    <comment ref="B4" authorId="0" shapeId="0">
+      <text>
+        <t>Formaat: 123456789L01. Staat op uw aangifte loonheffingen of in uw portaal bij de Belastingdienst.</t>
+      </text>
+    </comment>
+    <comment ref="B5" authorId="0" shapeId="0">
+      <text>
+        <t>Kies de sector waarin uw bedrijf is ingedeeld. Bij twijfel: zie de sectorbeschikking van de Belastingdienst.</t>
+      </text>
+    </comment>
+    <comment ref="B6" authorId="0" shapeId="0">
+      <text>
+        <t>Klein: minder dan 25 werknemers. Middel: 25 - 100 werknemers. Groot: meer dan 100 werknemers. Bij twijfel: leeglaten, wij bepalen dit.</t>
+      </text>
+    </comment>
+    <comment ref="B7" authorId="0" shapeId="0">
+      <text>
+        <t>Optioneel. De 4-cijferige code van uw CAO volgens het CBS. Bij geen CAO: leeglaten.</t>
+      </text>
+    </comment>
+    <comment ref="B8" authorId="0" shapeId="0">
+      <text>
+        <t>WBSO = Wet Bevordering Speur- en Ontwikkelingswerk. Alleen 'Ja' als u een WBSO-beschikking van RVO heeft.</t>
       </text>
     </comment>
   </commentList>
@@ -773,7 +873,7 @@
         </is>
       </c>
       <c r="B21" s="10">
-        <f>COUNTA('1. Bedrijf &amp; Contact'!$B$4,'1. Bedrijf &amp; Contact'!$B$5,'1. Bedrijf &amp; Contact'!$B$6,'1. Bedrijf &amp; Contact'!$B$7,'1. Bedrijf &amp; Contact'!$B$12,'1. Bedrijf &amp; Contact'!$B$14,'1. Bedrijf &amp; Contact'!$B$15,'1. Bedrijf &amp; Contact'!$B$18,'1. Bedrijf &amp; Contact'!$B$20,'1. Bedrijf &amp; Contact'!$B$21,'1. Bedrijf &amp; Contact'!$B$24)&amp;" / 11"</f>
+        <f>COUNTA('1. Bedrijf &amp; Contact'!$B$4,'1. Bedrijf &amp; Contact'!$B$5,'1. Bedrijf &amp; Contact'!$B$6,'1. Bedrijf &amp; Contact'!$B$7,'1. Bedrijf &amp; Contact'!$B$12,'1. Bedrijf &amp; Contact'!$B$14,'1. Bedrijf &amp; Contact'!$B$15,'1. Bedrijf &amp; Contact'!$B$18,'1. Bedrijf &amp; Contact'!$B$20,'1. Bedrijf &amp; Contact'!$B$21,'1. Bedrijf &amp; Contact'!$B$24,'2. Payroll basis'!$B$4,'2. Payroll basis'!$B$8,'2. Payroll basis'!$B$12,'2. Payroll basis'!$B$15,'2. Payroll basis'!$B$16,'2. Payroll basis'!$B$17,'2. Payroll basis'!$B$21,'2. Payroll basis'!$B$25,'2. Payroll basis'!$B$26,'3. Loonheffing'!$B$4,'3. Loonheffing'!$B$5,'3. Loonheffing'!$B$6,'3. Loonheffing'!$B$8)&amp;" / 24"</f>
         <v/>
       </c>
       <c r="C21" s="11" t="inlineStr">
@@ -789,7 +889,7 @@
         </is>
       </c>
       <c r="B22" s="10">
-        <f>IFERROR(TEXT(COUNTA('1. Bedrijf &amp; Contact'!$B$4,'1. Bedrijf &amp; Contact'!$B$5,'1. Bedrijf &amp; Contact'!$B$6,'1. Bedrijf &amp; Contact'!$B$7,'1. Bedrijf &amp; Contact'!$B$12,'1. Bedrijf &amp; Contact'!$B$14,'1. Bedrijf &amp; Contact'!$B$15,'1. Bedrijf &amp; Contact'!$B$18,'1. Bedrijf &amp; Contact'!$B$20,'1. Bedrijf &amp; Contact'!$B$21,'1. Bedrijf &amp; Contact'!$B$24)/11,"0%"),"0%")</f>
+        <f>IFERROR(TEXT(COUNTA('1. Bedrijf &amp; Contact'!$B$4,'1. Bedrijf &amp; Contact'!$B$5,'1. Bedrijf &amp; Contact'!$B$6,'1. Bedrijf &amp; Contact'!$B$7,'1. Bedrijf &amp; Contact'!$B$12,'1. Bedrijf &amp; Contact'!$B$14,'1. Bedrijf &amp; Contact'!$B$15,'1. Bedrijf &amp; Contact'!$B$18,'1. Bedrijf &amp; Contact'!$B$20,'1. Bedrijf &amp; Contact'!$B$21,'1. Bedrijf &amp; Contact'!$B$24,'2. Payroll basis'!$B$4,'2. Payroll basis'!$B$8,'2. Payroll basis'!$B$12,'2. Payroll basis'!$B$15,'2. Payroll basis'!$B$16,'2. Payroll basis'!$B$17,'2. Payroll basis'!$B$21,'2. Payroll basis'!$B$25,'2. Payroll basis'!$B$26,'3. Loonheffing'!$B$4,'3. Loonheffing'!$B$5,'3. Loonheffing'!$B$6,'3. Loonheffing'!$B$8)/24,"0%"),"0%")</f>
         <v/>
       </c>
     </row>
@@ -1071,7 +1171,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -1091,14 +1191,267 @@
         </is>
       </c>
     </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>CAO (Collectieve arbeidsovereenkomst)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="13" t="inlineStr">
+        <is>
+          <t>Is een CAO van toepassing? *</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>Zo ja, welke CAO?</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="n"/>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Werktijden (standaard fulltime)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="13" t="inlineStr">
+        <is>
+          <t>Uren per week *</t>
+        </is>
+      </c>
+      <c r="B8" s="14" t="n">
+        <v>40</v>
+      </c>
+      <c r="C8" s="15" t="inlineStr">
+        <is>
+          <t>ma</t>
+        </is>
+      </c>
+      <c r="D8" s="15" t="inlineStr">
+        <is>
+          <t>di</t>
+        </is>
+      </c>
+      <c r="E8" s="15" t="inlineStr">
+        <is>
+          <t>wo</t>
+        </is>
+      </c>
+      <c r="F8" s="15" t="inlineStr">
+        <is>
+          <t>do</t>
+        </is>
+      </c>
+      <c r="G8" s="15" t="inlineStr">
+        <is>
+          <t>vr</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>Uren per dag (maandag - vrijdag)</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="D9" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="E9" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="F9" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="G9" s="8" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Salarisperiode</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="13" t="inlineStr">
+        <is>
+          <t>Salarisperiode *</t>
+        </is>
+      </c>
+      <c r="B12" s="14" t="inlineStr">
+        <is>
+          <t>Maand</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Salarisstrook</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="13" t="inlineStr">
+        <is>
+          <t>Taal salarisstrook *</t>
+        </is>
+      </c>
+      <c r="B15" s="14" t="inlineStr">
+        <is>
+          <t>Nederlands</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="13" t="inlineStr">
+        <is>
+          <t>Logo van uw bedrijf op salarisstrook? *</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="13" t="inlineStr">
+        <is>
+          <t>Strook zichtbaar voor medewerker *</t>
+        </is>
+      </c>
+      <c r="B17" s="14" t="inlineStr">
+        <is>
+          <t>Op de betaaldatum</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>Aantal dagen na betaaldatum</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="n"/>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>30%-regeling (voor buitenlandse kenniswerkers)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="13" t="inlineStr">
+        <is>
+          <t>30%-regeling van toepassing? *</t>
+        </is>
+      </c>
+      <c r="B21" s="14" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>Aantal medewerkers met 30%-regeling</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="n"/>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Overige werknemerstypen</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="13" t="inlineStr">
+        <is>
+          <t>Stagiaires in dienst? *</t>
+        </is>
+      </c>
+      <c r="B25" s="14" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="13" t="inlineStr">
+        <is>
+          <t>Oproepkrachten in dienst? *</t>
+        </is>
+      </c>
+      <c r="B26" s="14" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="22" customHeight="1">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Opmerkingen</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="12" t="n"/>
+    </row>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
-  <mergeCells count="1">
+  <mergeCells count="9">
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A7:H7"/>
+    <mergeCell ref="A20:H20"/>
+    <mergeCell ref="A24:H24"/>
+    <mergeCell ref="A29:H32"/>
+    <mergeCell ref="A28:H28"/>
+    <mergeCell ref="A11:H11"/>
+    <mergeCell ref="A14:H14"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
+  <dataValidations count="6">
+    <dataValidation sqref="B4 B16 B25" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ongeldige invoer" error="Ongeldige keuze. Kies uit de lijst." type="list">
+      <formula1>=val_JaNee</formula1>
+    </dataValidation>
+    <dataValidation sqref="B12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ongeldige invoer" error="Ongeldige keuze. Kies uit de lijst." type="list">
+      <formula1>=val_Salarisperiode</formula1>
+    </dataValidation>
+    <dataValidation sqref="B15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ongeldige invoer" error="Ongeldige keuze. Kies uit de lijst." type="list">
+      <formula1>=val_Taal</formula1>
+    </dataValidation>
+    <dataValidation sqref="B17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ongeldige invoer" error="Ongeldige keuze. Kies uit de lijst." type="list">
+      <formula1>=val_Zichtbaarheid</formula1>
+    </dataValidation>
+    <dataValidation sqref="B21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ongeldige invoer" error="Ongeldige keuze. Kies uit de lijst." type="list">
+      <formula1>=val_30pct</formula1>
+    </dataValidation>
+    <dataValidation sqref="B26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ongeldige invoer" error="Ongeldige keuze. Kies uit de lijst." type="list">
+      <formula1>=val_Oproep</formula1>
+    </dataValidation>
+  </dataValidations>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -1108,7 +1461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -1128,14 +1481,114 @@
         </is>
       </c>
     </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Gegevens aangifte loonheffingen</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="13" t="inlineStr">
+        <is>
+          <t>Loonheffingsnummer *</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>Sector (sectorindeling Belastingdienst) *</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="13" t="inlineStr">
+        <is>
+          <t>Indeling werkgever *</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>CBS CAO-code</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="13" t="inlineStr">
+        <is>
+          <t>WBSO-subsidie van toepassing? *</t>
+        </is>
+      </c>
+      <c r="B8" s="14" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>WHK-premie (gedifferentieerde premie Werkhervattingskas)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="16" t="inlineStr">
+        <is>
+          <t>U hoeft hier GEEN premiepercentages in te vullen.
+Stuur de WHK-beschikking van de Belastingdienst voor het lopende jaar mee als bijlage (zie de bijlagen-checklist op het tabblad 'Start').
+Wij verwerken op basis van die beschikking de WGA-premie, ZW-premie en eventueel eigenrisicodragerschap in de inrichting.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Opmerkingen</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="12" t="n"/>
+    </row>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
-  <mergeCells count="1">
+  <mergeCells count="6">
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A17:H20"/>
+    <mergeCell ref="A16:H16"/>
+    <mergeCell ref="A11:H14"/>
+    <mergeCell ref="A10:H10"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
+  <dataValidations count="3">
+    <dataValidation sqref="B5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ongeldige invoer" error="Ongeldige keuze. Kies uit de lijst." type="list">
+      <formula1>=val_Sector</formula1>
+    </dataValidation>
+    <dataValidation sqref="B6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ongeldige invoer" error="Ongeldige keuze. Kies uit de lijst." type="list">
+      <formula1>=val_Indeling</formula1>
+    </dataValidation>
+    <dataValidation sqref="B8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ongeldige invoer" error="Ongeldige keuze. Kies uit de lijst." type="list">
+      <formula1>=val_JaNee</formula1>
+    </dataValidation>
+  </dataValidations>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -1276,72 +1729,72 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="14" t="inlineStr">
+      <c r="A1" s="17" t="inlineStr">
         <is>
           <t>val_JaNee</t>
         </is>
       </c>
-      <c r="B1" s="14" t="inlineStr">
+      <c r="B1" s="17" t="inlineStr">
         <is>
           <t>val_Salarisperiode</t>
         </is>
       </c>
-      <c r="C1" s="14" t="inlineStr">
+      <c r="C1" s="17" t="inlineStr">
         <is>
           <t>val_Taal</t>
         </is>
       </c>
-      <c r="D1" s="14" t="inlineStr">
+      <c r="D1" s="17" t="inlineStr">
         <is>
           <t>val_Indeling</t>
         </is>
       </c>
-      <c r="E1" s="14" t="inlineStr">
+      <c r="E1" s="17" t="inlineStr">
         <is>
           <t>val_Oproep</t>
         </is>
       </c>
-      <c r="F1" s="14" t="inlineStr">
+      <c r="F1" s="17" t="inlineStr">
         <is>
           <t>val_Maand</t>
         </is>
       </c>
-      <c r="G1" s="14" t="inlineStr">
+      <c r="G1" s="17" t="inlineStr">
         <is>
           <t>val_Zichtbaarheid</t>
         </is>
       </c>
-      <c r="H1" s="14" t="inlineStr">
+      <c r="H1" s="17" t="inlineStr">
         <is>
           <t>val_Formaat</t>
         </is>
       </c>
-      <c r="I1" s="14" t="inlineStr">
+      <c r="I1" s="17" t="inlineStr">
         <is>
           <t>val_Basisperiode</t>
         </is>
       </c>
-      <c r="J1" s="14" t="inlineStr">
+      <c r="J1" s="17" t="inlineStr">
         <is>
           <t>val_FinSysteem</t>
         </is>
       </c>
-      <c r="K1" s="14" t="inlineStr">
+      <c r="K1" s="17" t="inlineStr">
         <is>
           <t>val_30pct</t>
         </is>
       </c>
-      <c r="L1" s="14" t="inlineStr">
+      <c r="L1" s="17" t="inlineStr">
         <is>
           <t>val_Toggle</t>
         </is>
       </c>
-      <c r="M1" s="14" t="inlineStr">
+      <c r="M1" s="17" t="inlineStr">
         <is>
           <t>val_Checkbox</t>
         </is>
       </c>
-      <c r="N1" s="14" t="inlineStr">
+      <c r="N1" s="17" t="inlineStr">
         <is>
           <t>val_Sector</t>
         </is>

</xml_diff>

<commit_message>
Phase 5: Reserveringen, Verlof/GL and Akkoord sheets
Reserveringen & Pensioen: vakantiegeld (8,33% / Juni-Mei
defaults), 13th month, BPF yes/no with two clearly separated
branches (BPF: fund name + number; non-BPF: premiums, franchise,
max, age limits), supplementary schemes yes/no, Advanced IKB
toggle with grey-fill IKB input cells.
Verlof & Grootboek: WAZO table (7 rows x 3 cols, statutory
minimum defaults), GL block (financial system, format, per cost
center), GL schema attachment reference.
Akkoord: client, signer + function, date, signature row,
2 acceptance dropdowns.
36 required fields, 0 formula errors, 29.5 KB.

https://claude.ai/code/session_01QG7xshNkELyspBZLGsyRFs
</commit_message>
<xml_diff>
--- a/outputs/Payroll_Discovery_Document_MKB.xlsx
+++ b/outputs/Payroll_Discovery_Document_MKB.xlsx
@@ -39,7 +39,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -87,6 +87,18 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00C00000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F3864"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F3864"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -149,7 +161,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -195,6 +207,16 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -413,6 +435,121 @@
     <comment ref="B8" authorId="0" shapeId="0">
       <text>
         <t>WBSO = Wet Bevordering Speur- en Ontwikkelingswerk. Alleen 'Ja' als u een WBSO-beschikking van RVO heeft.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment5.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>SD Worx</author>
+  </authors>
+  <commentList>
+    <comment ref="B4" authorId="0" shapeId="0">
+      <text>
+        <t>Wettelijk minimum 8,00%. In veel CAO's 8,33% (= 1 maand extra salaris).</t>
+      </text>
+    </comment>
+    <comment ref="B11" authorId="0" shapeId="0">
+      <text>
+        <t>Alleen invullen als '13e maand van toepassing' = Ja. Meestal december.</t>
+      </text>
+    </comment>
+    <comment ref="B14" authorId="0" shapeId="0">
+      <text>
+        <t>BPF = verplicht pensioenfonds per branche (bv. PFZW, BPF Bouw, BPF Metaal). Bij 'Ja' volgt alles uit het BPF-reglement. Bij 'Nee' heeft u een eigen regeling.</t>
+      </text>
+    </comment>
+    <comment ref="B17" authorId="0" shapeId="0">
+      <text>
+        <t>Bijv. 'PFZW', 'BPF Metaal en Techniek', 'BPF Bouw'.</t>
+      </text>
+    </comment>
+    <comment ref="B23" authorId="0" shapeId="0">
+      <text>
+        <t>Bedrag waarover GEEN pensioen wordt opgebouwd. Bij BPF: leeglaten. Bij twijfel: vraag uw pensioenadviseur.</t>
+      </text>
+    </comment>
+    <comment ref="B24" authorId="0" shapeId="0">
+      <text>
+        <t>Wettelijk maximum 2025: circa EUR 137.800. Laat leeg voor 'geen maximum'.</t>
+      </text>
+    </comment>
+    <comment ref="B26" authorId="0" shapeId="0">
+      <text>
+        <t>Standaard tot AOW-leeftijd. Wijzig alleen als uw regeling anders bepaalt.</t>
+      </text>
+    </comment>
+    <comment ref="B29" authorId="0" shapeId="0">
+      <text>
+        <t>Denk aan WGA-hiaatverzekering, pensioen-excedent, netto pensioen, WIA-bodem. Bij 'Ja': uw consultant neemt dit mondeling met u door. Wij vragen hier geen details.</t>
+      </text>
+    </comment>
+    <comment ref="B32" authorId="0" shapeId="0">
+      <text>
+        <t>Kies 'Uitgebreid' als u een IKB-regeling heeft. Kies 'Basis' om IKB-velden te negeren.</t>
+      </text>
+    </comment>
+    <comment ref="B33" authorId="0" shapeId="0">
+      <text>
+        <t>Alleen invullen bij toggle = 'Uitgebreid'.</t>
+      </text>
+    </comment>
+    <comment ref="B34" authorId="0" shapeId="0">
+      <text>
+        <t>Alleen invullen bij toggle = 'Uitgebreid'.</t>
+      </text>
+    </comment>
+    <comment ref="B35" authorId="0" shapeId="0">
+      <text>
+        <t>Alleen invullen bij toggle = 'Uitgebreid'.</t>
+      </text>
+    </comment>
+    <comment ref="B36" authorId="0" shapeId="0">
+      <text>
+        <t>Alleen invullen bij toggle = 'Uitgebreid'.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment6.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>SD Worx</author>
+  </authors>
+  <commentList>
+    <comment ref="B16" authorId="0" shapeId="0">
+      <text>
+        <t>Kies uw financiele pakket. Kies 'Anders' als uw pakket er niet bij staat - wij nemen dan contact op.</t>
+      </text>
+    </comment>
+    <comment ref="B17" authorId="0" shapeId="0">
+      <text>
+        <t>Meestgebruikt: CSV of XML. Exact Online: XML. AFAS: XML of CSV.</t>
+      </text>
+    </comment>
+    <comment ref="B18" authorId="0" shapeId="0">
+      <text>
+        <t>Kies 'Ja' als u per afdeling / kostenplaats gesplitste boekingen wilt.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment7.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>SD Worx</author>
+  </authors>
+  <commentList>
+    <comment ref="B11" authorId="0" shapeId="0">
+      <text>
+        <t>Formaat: DD-MM-JJJJ</t>
       </text>
     </comment>
   </commentList>
@@ -873,7 +1010,7 @@
         </is>
       </c>
       <c r="B21" s="10">
-        <f>COUNTA('1. Bedrijf &amp; Contact'!$B$4,'1. Bedrijf &amp; Contact'!$B$5,'1. Bedrijf &amp; Contact'!$B$6,'1. Bedrijf &amp; Contact'!$B$7,'1. Bedrijf &amp; Contact'!$B$12,'1. Bedrijf &amp; Contact'!$B$14,'1. Bedrijf &amp; Contact'!$B$15,'1. Bedrijf &amp; Contact'!$B$18,'1. Bedrijf &amp; Contact'!$B$20,'1. Bedrijf &amp; Contact'!$B$21,'1. Bedrijf &amp; Contact'!$B$24,'2. Payroll basis'!$B$4,'2. Payroll basis'!$B$8,'2. Payroll basis'!$B$12,'2. Payroll basis'!$B$15,'2. Payroll basis'!$B$16,'2. Payroll basis'!$B$17,'2. Payroll basis'!$B$21,'2. Payroll basis'!$B$25,'2. Payroll basis'!$B$26,'3. Loonheffing'!$B$4,'3. Loonheffing'!$B$5,'3. Loonheffing'!$B$6,'3. Loonheffing'!$B$8)&amp;" / 24"</f>
+        <f>COUNTA('1. Bedrijf &amp; Contact'!$B$4,'1. Bedrijf &amp; Contact'!$B$5,'1. Bedrijf &amp; Contact'!$B$6,'1. Bedrijf &amp; Contact'!$B$7,'1. Bedrijf &amp; Contact'!$B$12,'1. Bedrijf &amp; Contact'!$B$14,'1. Bedrijf &amp; Contact'!$B$15,'1. Bedrijf &amp; Contact'!$B$18,'1. Bedrijf &amp; Contact'!$B$20,'1. Bedrijf &amp; Contact'!$B$21,'1. Bedrijf &amp; Contact'!$B$24,'2. Payroll basis'!$B$4,'2. Payroll basis'!$B$8,'2. Payroll basis'!$B$12,'2. Payroll basis'!$B$15,'2. Payroll basis'!$B$16,'2. Payroll basis'!$B$17,'2. Payroll basis'!$B$21,'2. Payroll basis'!$B$25,'2. Payroll basis'!$B$26,'3. Loonheffing'!$B$4,'3. Loonheffing'!$B$5,'3. Loonheffing'!$B$6,'3. Loonheffing'!$B$8,'4. Reserveringen &amp; Pensioen'!$B$10,'4. Reserveringen &amp; Pensioen'!$B$14,'4. Reserveringen &amp; Pensioen'!$B$29,'5. Verlof &amp; Grootboek'!$B$16,'5. Verlof &amp; Grootboek'!$B$17,'5. Verlof &amp; Grootboek'!$B$18,'6. Akkoord'!$B$8,'6. Akkoord'!$B$9,'6. Akkoord'!$B$11,'6. Akkoord'!$B$12,'6. Akkoord'!$B$15,'6. Akkoord'!$B$16)&amp;" / 36"</f>
         <v/>
       </c>
       <c r="C21" s="11" t="inlineStr">
@@ -889,7 +1026,7 @@
         </is>
       </c>
       <c r="B22" s="10">
-        <f>IFERROR(TEXT(COUNTA('1. Bedrijf &amp; Contact'!$B$4,'1. Bedrijf &amp; Contact'!$B$5,'1. Bedrijf &amp; Contact'!$B$6,'1. Bedrijf &amp; Contact'!$B$7,'1. Bedrijf &amp; Contact'!$B$12,'1. Bedrijf &amp; Contact'!$B$14,'1. Bedrijf &amp; Contact'!$B$15,'1. Bedrijf &amp; Contact'!$B$18,'1. Bedrijf &amp; Contact'!$B$20,'1. Bedrijf &amp; Contact'!$B$21,'1. Bedrijf &amp; Contact'!$B$24,'2. Payroll basis'!$B$4,'2. Payroll basis'!$B$8,'2. Payroll basis'!$B$12,'2. Payroll basis'!$B$15,'2. Payroll basis'!$B$16,'2. Payroll basis'!$B$17,'2. Payroll basis'!$B$21,'2. Payroll basis'!$B$25,'2. Payroll basis'!$B$26,'3. Loonheffing'!$B$4,'3. Loonheffing'!$B$5,'3. Loonheffing'!$B$6,'3. Loonheffing'!$B$8)/24,"0%"),"0%")</f>
+        <f>IFERROR(TEXT(COUNTA('1. Bedrijf &amp; Contact'!$B$4,'1. Bedrijf &amp; Contact'!$B$5,'1. Bedrijf &amp; Contact'!$B$6,'1. Bedrijf &amp; Contact'!$B$7,'1. Bedrijf &amp; Contact'!$B$12,'1. Bedrijf &amp; Contact'!$B$14,'1. Bedrijf &amp; Contact'!$B$15,'1. Bedrijf &amp; Contact'!$B$18,'1. Bedrijf &amp; Contact'!$B$20,'1. Bedrijf &amp; Contact'!$B$21,'1. Bedrijf &amp; Contact'!$B$24,'2. Payroll basis'!$B$4,'2. Payroll basis'!$B$8,'2. Payroll basis'!$B$12,'2. Payroll basis'!$B$15,'2. Payroll basis'!$B$16,'2. Payroll basis'!$B$17,'2. Payroll basis'!$B$21,'2. Payroll basis'!$B$25,'2. Payroll basis'!$B$26,'3. Loonheffing'!$B$4,'3. Loonheffing'!$B$5,'3. Loonheffing'!$B$6,'3. Loonheffing'!$B$8,'4. Reserveringen &amp; Pensioen'!$B$10,'4. Reserveringen &amp; Pensioen'!$B$14,'4. Reserveringen &amp; Pensioen'!$B$29,'5. Verlof &amp; Grootboek'!$B$16,'5. Verlof &amp; Grootboek'!$B$17,'5. Verlof &amp; Grootboek'!$B$18,'6. Akkoord'!$B$8,'6. Akkoord'!$B$9,'6. Akkoord'!$B$11,'6. Akkoord'!$B$12,'6. Akkoord'!$B$15,'6. Akkoord'!$B$16)/36,"0%"),"0%")</f>
         <v/>
       </c>
     </row>
@@ -1598,7 +1735,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -1618,14 +1755,297 @@
         </is>
       </c>
     </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Vakantiegeld</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Uitbetalingspercentage</t>
+        </is>
+      </c>
+      <c r="B4" s="14" t="inlineStr">
+        <is>
+          <t>8,33%</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>Referentieperiode van</t>
+        </is>
+      </c>
+      <c r="B5" s="14" t="inlineStr">
+        <is>
+          <t>Juni</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Referentieperiode tot en met</t>
+        </is>
+      </c>
+      <c r="B6" s="14" t="inlineStr">
+        <is>
+          <t>Mei</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>Uitbetaalmaand</t>
+        </is>
+      </c>
+      <c r="B7" s="14" t="inlineStr">
+        <is>
+          <t>Mei</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>13e maand</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="13" t="inlineStr">
+        <is>
+          <t>13e maand van toepassing? *</t>
+        </is>
+      </c>
+      <c r="B10" s="14" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>Uitbetaalmaand 13e maand</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="n"/>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Pensioen</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="13" t="inlineStr">
+        <is>
+          <t>Aangesloten bij bedrijfstakpensioenfonds (BPF)? *</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>Bij BPF = Ja</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>Naam bedrijfstakpensioenfonds</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>Aansluitingsnummer bij het fonds</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="17" t="inlineStr">
+        <is>
+          <t>Bij BPF = Nee (eigen pensioenregeling)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>Premie werknemer (%)</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>Premie werkgever (%)</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>Franchise (EUR per jaar)</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>Maximum pensioengevend jaarloon (EUR)</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>Minimum leeftijd voor pensioenopbouw</t>
+        </is>
+      </c>
+      <c r="B25" s="14" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>Maximum leeftijd voor pensioenopbouw</t>
+        </is>
+      </c>
+      <c r="B26" s="14" t="inlineStr">
+        <is>
+          <t>AOW-leeftijd</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="22" customHeight="1">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Aanvullende regelingen</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="13" t="inlineStr">
+        <is>
+          <t>Heeft u aanvullende regelingen? *</t>
+        </is>
+      </c>
+      <c r="B29" s="14" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="22" customHeight="1">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Geavanceerd (optioneel) - Individueel Keuzebudget (IKB)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>IKB-toggle</t>
+        </is>
+      </c>
+      <c r="B32" s="14" t="inlineStr">
+        <is>
+          <t>Basis</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="inlineStr">
+        <is>
+          <t>IKB-percentage</t>
+        </is>
+      </c>
+      <c r="B33" s="14" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="inlineStr">
+        <is>
+          <t>IKB-referentieperiode van</t>
+        </is>
+      </c>
+      <c r="B34" s="14" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="6" t="inlineStr">
+        <is>
+          <t>IKB-referentieperiode tot en met</t>
+        </is>
+      </c>
+      <c r="B35" s="14" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <t>IKB-uitbetaalmaand</t>
+        </is>
+      </c>
+      <c r="B36" s="14" t="n"/>
+    </row>
+    <row r="38" ht="22" customHeight="1">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>Opmerkingen</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="12" t="n"/>
+    </row>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
-  <mergeCells count="1">
+  <mergeCells count="8">
+    <mergeCell ref="A9:H9"/>
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A38:H38"/>
+    <mergeCell ref="A39:H42"/>
+    <mergeCell ref="A28:H28"/>
+    <mergeCell ref="A13:H13"/>
     <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A31:H31"/>
   </mergeCells>
+  <dataValidations count="3">
+    <dataValidation sqref="B7 B11 B36" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ongeldige invoer" error="Ongeldige keuze. Kies uit de lijst." type="list">
+      <formula1>=val_Maand</formula1>
+    </dataValidation>
+    <dataValidation sqref="B10 B14 B29" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ongeldige invoer" error="Ongeldige keuze. Kies uit de lijst." type="list">
+      <formula1>=val_JaNee</formula1>
+    </dataValidation>
+    <dataValidation sqref="B32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ongeldige invoer" error="Ongeldige keuze. Kies uit de lijst." type="list">
+      <formula1>=val_Toggle</formula1>
+    </dataValidation>
+  </dataValidations>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -1635,7 +2055,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -1655,14 +2075,264 @@
         </is>
       </c>
     </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Wettelijke verlofregelingen (WAZO)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="18" t="inlineStr">
+        <is>
+          <t>Soort verlof</t>
+        </is>
+      </c>
+      <c r="B4" s="18" t="inlineStr">
+        <is>
+          <t>Doorbetaald %</t>
+        </is>
+      </c>
+      <c r="C4" s="18" t="inlineStr">
+        <is>
+          <t>Pensioenopbouw</t>
+        </is>
+      </c>
+      <c r="D4" s="18" t="inlineStr">
+        <is>
+          <t>Vakantiegeld-opbouw</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="19" t="inlineStr">
+        <is>
+          <t>Geboorteverlof (1 week)</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="19" t="inlineStr">
+        <is>
+          <t>Aanvullend geboorteverlof (5 weken)</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="n">
+        <v>70</v>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="19" t="inlineStr">
+        <is>
+          <t>Betaald ouderschapsverlof (9 weken)</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="n">
+        <v>70</v>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="19" t="inlineStr">
+        <is>
+          <t>Onbetaald ouderschapsverlof</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="19" t="inlineStr">
+        <is>
+          <t>Kortdurend zorgverlof</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="n">
+        <v>70</v>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="19" t="inlineStr">
+        <is>
+          <t>Langdurig zorgverlof</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="19" t="inlineStr">
+        <is>
+          <t>Onbetaald verlof (algemeen)</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Defaults = wettelijk minimum. Overschrijf indien uw CAO gunstigere voorwaarden biedt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Grootboek-export (journaalpost)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="13" t="inlineStr">
+        <is>
+          <t>Financieel systeem *</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="13" t="inlineStr">
+        <is>
+          <t>Bestandsformaat export *</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="13" t="inlineStr">
+        <is>
+          <t>Journaalpost per kostenplaats splitsen? *</t>
+        </is>
+      </c>
+      <c r="B18" s="14" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="16" t="inlineStr">
+        <is>
+          <t>Stuur uw GROOTBOEKSCHEMA + een recente JOURNAALPOST als bijlage mee (zie bijlagen-checklist op Start). Wij mappen uw looncomponenten hieraan - u hoeft hier geen aparte kolommen op te geven.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Opmerkingen</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="12" t="n"/>
+    </row>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
-  <mergeCells count="1">
+  <mergeCells count="6">
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A15:H15"/>
+    <mergeCell ref="A24:H24"/>
+    <mergeCell ref="A20:H22"/>
+    <mergeCell ref="A25:H28"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
+  <dataValidations count="3">
+    <dataValidation sqref="B18 C5 C6 C7 C8 C9 C10 C11 D5 D6 D7 D8 D9 D10 D11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ongeldige invoer" error="Ongeldige keuze. Kies uit de lijst." type="list">
+      <formula1>=val_JaNee</formula1>
+    </dataValidation>
+    <dataValidation sqref="B16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ongeldige invoer" error="Ongeldige keuze. Kies uit de lijst." type="list">
+      <formula1>=val_FinSysteem</formula1>
+    </dataValidation>
+    <dataValidation sqref="B17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ongeldige invoer" error="Ongeldige keuze. Kies uit de lijst." type="list">
+      <formula1>=val_Formaat</formula1>
+    </dataValidation>
+  </dataValidations>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -1672,7 +2342,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -1692,14 +2362,117 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="20" t="inlineStr">
+        <is>
+          <t>Hierbij verklaart ondergetekende dat de inrichting van Cobra conform de gegevens in dit inventarisatiedocument is uitgevoerd en geeft akkoord op de onderstaande punten.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4"/>
+    <row r="5"/>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Ondertekening</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="13" t="inlineStr">
+        <is>
+          <t>Naam klant / bedrijf *</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="13" t="inlineStr">
+        <is>
+          <t>Naam ondertekenaar (contactpersoon) *</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>Functie ondertekenaar</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t>Datum *</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="n"/>
+    </row>
+    <row r="12" ht="60" customHeight="1">
+      <c r="A12" s="13" t="inlineStr">
+        <is>
+          <t>Handtekening *</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="n"/>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Akkoordverklaringen</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="13" t="inlineStr">
+        <is>
+          <t>Akkoord met de Cobra-setup zoals beschreven in dit document *</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="13" t="inlineStr">
+        <is>
+          <t>Akkoord met de schaduwverwerking(en) *</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="n"/>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Opmerkingen</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="12" t="n"/>
+    </row>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
-  <mergeCells count="1">
+  <mergeCells count="6">
+    <mergeCell ref="A18:H18"/>
+    <mergeCell ref="A7:H7"/>
+    <mergeCell ref="A3:H5"/>
+    <mergeCell ref="A14:H14"/>
     <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A19:H22"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="B15 B16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ongeldige invoer" error="Ongeldige keuze. Kies uit de lijst." type="list">
+      <formula1>=val_JaNee</formula1>
+    </dataValidation>
+  </dataValidations>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -1729,72 +2502,72 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="17" t="inlineStr">
+      <c r="A1" s="21" t="inlineStr">
         <is>
           <t>val_JaNee</t>
         </is>
       </c>
-      <c r="B1" s="17" t="inlineStr">
+      <c r="B1" s="21" t="inlineStr">
         <is>
           <t>val_Salarisperiode</t>
         </is>
       </c>
-      <c r="C1" s="17" t="inlineStr">
+      <c r="C1" s="21" t="inlineStr">
         <is>
           <t>val_Taal</t>
         </is>
       </c>
-      <c r="D1" s="17" t="inlineStr">
+      <c r="D1" s="21" t="inlineStr">
         <is>
           <t>val_Indeling</t>
         </is>
       </c>
-      <c r="E1" s="17" t="inlineStr">
+      <c r="E1" s="21" t="inlineStr">
         <is>
           <t>val_Oproep</t>
         </is>
       </c>
-      <c r="F1" s="17" t="inlineStr">
+      <c r="F1" s="21" t="inlineStr">
         <is>
           <t>val_Maand</t>
         </is>
       </c>
-      <c r="G1" s="17" t="inlineStr">
+      <c r="G1" s="21" t="inlineStr">
         <is>
           <t>val_Zichtbaarheid</t>
         </is>
       </c>
-      <c r="H1" s="17" t="inlineStr">
+      <c r="H1" s="21" t="inlineStr">
         <is>
           <t>val_Formaat</t>
         </is>
       </c>
-      <c r="I1" s="17" t="inlineStr">
+      <c r="I1" s="21" t="inlineStr">
         <is>
           <t>val_Basisperiode</t>
         </is>
       </c>
-      <c r="J1" s="17" t="inlineStr">
+      <c r="J1" s="21" t="inlineStr">
         <is>
           <t>val_FinSysteem</t>
         </is>
       </c>
-      <c r="K1" s="17" t="inlineStr">
+      <c r="K1" s="21" t="inlineStr">
         <is>
           <t>val_30pct</t>
         </is>
       </c>
-      <c r="L1" s="17" t="inlineStr">
+      <c r="L1" s="21" t="inlineStr">
         <is>
           <t>val_Toggle</t>
         </is>
       </c>
-      <c r="M1" s="17" t="inlineStr">
+      <c r="M1" s="21" t="inlineStr">
         <is>
           <t>val_Checkbox</t>
         </is>
       </c>
-      <c r="N1" s="17" t="inlineStr">
+      <c r="N1" s="21" t="inlineStr">
         <is>
           <t>val_Sector</t>
         </is>

</xml_diff>

<commit_message>
Apply SD Worx branding and refine layout
- Embed SD Worx primary logo in the header of every sheet (PNG
  converted from the supplied PDF brand asset; auto-cropped and
  scaled to 190x63 px).
- Rework header: white background, right-aligned navy title next
  to logo, followed by a 4-px brand-yellow accent stripe instead
  of a solid dark header bar.
- Apply brand palette: navy #203040 (text), red #E01030 (required
  asterisk only, via rich text), yellow #F0B000 (stripe / left
  border of sub-headers), pale steel #E8ECF2 (sub-headers), warm
  cream #FFF4D1 (input cells), soft neutrals for defaults / help.
- Tighten layout: uniform 18pt row heights for content rows, 24pt
  for sub-headers, tighter print margins (0.4 / 0.5").
- 8/8 QA checks still pass; file size 199 KB (logo embedded per
  sheet), under the 500 KB budget.

https://claude.ai/code/session_01QG7xshNkELyspBZLGsyRFs
</commit_message>
<xml_diff>
--- a/outputs/Payroll_Discovery_Document_MKB.xlsx
+++ b/outputs/Payroll_Discovery_Document_MKB.xlsx
@@ -39,7 +39,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="11">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -50,8 +50,8 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="16"/>
+      <color rgb="00203040"/>
+      <sz val="18"/>
     </font>
     <font>
       <b val="1"/>
@@ -63,30 +63,25 @@
     </font>
     <font>
       <name val="Calibri"/>
+      <color rgb="00203040"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
       <i val="1"/>
-      <color rgb="007F7F7F"/>
+      <color rgb="006B7684"/>
       <sz val="9"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="001F3864"/>
+      <color rgb="00203040"/>
       <sz val="12"/>
     </font>
     <font>
       <name val="Calibri"/>
       <i val="1"/>
-      <color rgb="00595959"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00C00000"/>
+      <color rgb="005F6B7A"/>
       <sz val="11"/>
     </font>
     <font>
@@ -102,7 +97,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -111,31 +106,36 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F3864"/>
+        <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9E1F2"/>
+        <fgColor rgb="00F0B000"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="00E8ECF2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F2F2F2"/>
+        <fgColor rgb="00FFF4D1"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF8E7"/>
+        <fgColor rgb="00F4F5F7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF8E2"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -144,17 +144,22 @@
       <diagonal/>
     </border>
     <border>
+      <left style="thick">
+        <color rgb="00F0B000"/>
+      </left>
+    </border>
+    <border>
       <left style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="00C5CCD6"/>
       </left>
       <right style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="00C5CCD6"/>
       </right>
       <top style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="00C5CCD6"/>
       </top>
       <bottom style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="00C5CCD6"/>
       </bottom>
     </border>
   </borders>
@@ -164,53 +169,51 @@
   <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="right" vertical="center" indent="2"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
       <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -556,6 +559,216 @@
 </comments>
 </file>
 
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1809750" cy="600075"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1809750" cy="600075"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1809750" cy="600075"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1809750" cy="600075"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1809750" cy="600075"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1809750" cy="600075"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1809750" cy="600075"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -858,187 +1071,197 @@
     <col width="28" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
+    <row r="1" ht="55" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Payroll Discovery Document - MKB</t>
         </is>
       </c>
     </row>
+    <row r="2" ht="4" customHeight="1">
+      <c r="A2" s="2" t="n"/>
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+    </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Welkom! Dit document is de basis voor de inrichting van uw loonadministratie in Cobra (SD Worx).</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Vul per tabblad de gegevens in. Geschatte invultijd: 30 - 45 minuten. Velden met * zijn verplicht.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>Geel = door u in te vullen.   Lichtgrijs = voorstel (overschrijfbaar).   Bij twijfel: leeglaten en contact opnemen met uw consultant.</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
+    <row r="7" ht="24" customHeight="1">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>Uw contactpersoon bij SD Worx</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr">
+    <row r="8" ht="18" customHeight="1">
+      <c r="A8" s="7" t="inlineStr">
         <is>
           <t>Naam consultant</t>
         </is>
       </c>
-      <c r="B8" s="7" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="6" t="inlineStr">
+      <c r="B8" s="8" t="n"/>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
         <is>
           <t>E-mail</t>
         </is>
       </c>
-      <c r="B9" s="7" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="inlineStr">
+      <c r="B9" s="8" t="n"/>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="7" t="inlineStr">
         <is>
           <t>Telefoon</t>
         </is>
       </c>
-      <c r="B10" s="7" t="n"/>
-    </row>
-    <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="5" t="inlineStr">
+      <c r="B10" s="8" t="n"/>
+    </row>
+    <row r="12" ht="24" customHeight="1">
+      <c r="A12" s="6" t="inlineStr">
         <is>
           <t>Benodigde bijlagen  (aanvinken wat is meegestuurd)</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="inlineStr">
+      <c r="A13" s="9" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="B13" s="9" t="inlineStr">
+      <c r="B13" s="10" t="inlineStr">
         <is>
           <t>Kopie laatste loonstrook van ca. 5 medewerkers (incl. 1 met variabele beloning, 1 met pensioen)</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="inlineStr">
+      <c r="A14" s="9" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="B14" s="9" t="inlineStr">
+      <c r="B14" s="10" t="inlineStr">
         <is>
           <t>Kopie WHK-beschikking lopend jaar</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="inlineStr">
+      <c r="A15" s="9" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="B15" s="9" t="inlineStr">
+      <c r="B15" s="10" t="inlineStr">
         <is>
           <t>Kopie grootboekschema + laatste journaalpost (alleen als u GL-export wilt)</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="8" t="inlineStr">
+      <c r="A16" s="9" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="B16" s="9" t="inlineStr">
+      <c r="B16" s="10" t="inlineStr">
         <is>
           <t>Kopie pensioenregeling (alleen als u NIET bij een bedrijfstakpensioenfonds zit)</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="8" t="inlineStr">
+      <c r="A17" s="9" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="B17" s="9" t="inlineStr">
+      <c r="B17" s="10" t="inlineStr">
         <is>
           <t>CAO (alleen als van toepassing)</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="8" t="inlineStr">
+      <c r="A18" s="9" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="B18" s="9" t="inlineStr">
+      <c r="B18" s="10" t="inlineStr">
         <is>
           <t>Functielijst (functiecode + omschrijving)</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="22" customHeight="1">
-      <c r="A20" s="5" t="inlineStr">
+    <row r="20" ht="24" customHeight="1">
+      <c r="A20" s="6" t="inlineStr">
         <is>
           <t>Voortgang verplichte velden</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="6" t="inlineStr">
+    <row r="21" ht="18" customHeight="1">
+      <c r="A21" s="7" t="inlineStr">
         <is>
           <t>Aantal ingevuld / totaal</t>
         </is>
       </c>
-      <c r="B21" s="10">
+      <c r="B21" s="11">
         <f>COUNTA('1. Bedrijf &amp; Contact'!$B$4,'1. Bedrijf &amp; Contact'!$B$5,'1. Bedrijf &amp; Contact'!$B$6,'1. Bedrijf &amp; Contact'!$B$7,'1. Bedrijf &amp; Contact'!$B$12,'1. Bedrijf &amp; Contact'!$B$14,'1. Bedrijf &amp; Contact'!$B$15,'1. Bedrijf &amp; Contact'!$B$18,'1. Bedrijf &amp; Contact'!$B$20,'1. Bedrijf &amp; Contact'!$B$21,'1. Bedrijf &amp; Contact'!$B$24,'2. Payroll basis'!$B$4,'2. Payroll basis'!$B$8,'2. Payroll basis'!$B$12,'2. Payroll basis'!$B$15,'2. Payroll basis'!$B$16,'2. Payroll basis'!$B$17,'2. Payroll basis'!$B$21,'2. Payroll basis'!$B$25,'2. Payroll basis'!$B$26,'3. Loonheffing'!$B$4,'3. Loonheffing'!$B$5,'3. Loonheffing'!$B$6,'3. Loonheffing'!$B$8,'4. Reserveringen &amp; Pensioen'!$B$10,'4. Reserveringen &amp; Pensioen'!$B$14,'4. Reserveringen &amp; Pensioen'!$B$29,'5. Verlof &amp; Grootboek'!$B$16,'5. Verlof &amp; Grootboek'!$B$17,'5. Verlof &amp; Grootboek'!$B$18,'6. Akkoord'!$B$8,'6. Akkoord'!$B$9,'6. Akkoord'!$B$11,'6. Akkoord'!$B$12,'6. Akkoord'!$B$15,'6. Akkoord'!$B$16)&amp;" / 36"</f>
         <v/>
       </c>
-      <c r="C21" s="11" t="inlineStr">
+      <c r="C21" s="12" t="inlineStr">
         <is>
           <t>Tip: sla het bestand op of druk op F9 om de teller te verversen.</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="6" t="inlineStr">
+    <row r="22" ht="18" customHeight="1">
+      <c r="A22" s="7" t="inlineStr">
         <is>
           <t>Percentage ingevuld</t>
         </is>
       </c>
-      <c r="B22" s="10">
+      <c r="B22" s="11">
         <f>IFERROR(TEXT(COUNTA('1. Bedrijf &amp; Contact'!$B$4,'1. Bedrijf &amp; Contact'!$B$5,'1. Bedrijf &amp; Contact'!$B$6,'1. Bedrijf &amp; Contact'!$B$7,'1. Bedrijf &amp; Contact'!$B$12,'1. Bedrijf &amp; Contact'!$B$14,'1. Bedrijf &amp; Contact'!$B$15,'1. Bedrijf &amp; Contact'!$B$18,'1. Bedrijf &amp; Contact'!$B$20,'1. Bedrijf &amp; Contact'!$B$21,'1. Bedrijf &amp; Contact'!$B$24,'2. Payroll basis'!$B$4,'2. Payroll basis'!$B$8,'2. Payroll basis'!$B$12,'2. Payroll basis'!$B$15,'2. Payroll basis'!$B$16,'2. Payroll basis'!$B$17,'2. Payroll basis'!$B$21,'2. Payroll basis'!$B$25,'2. Payroll basis'!$B$26,'3. Loonheffing'!$B$4,'3. Loonheffing'!$B$5,'3. Loonheffing'!$B$6,'3. Loonheffing'!$B$8,'4. Reserveringen &amp; Pensioen'!$B$10,'4. Reserveringen &amp; Pensioen'!$B$14,'4. Reserveringen &amp; Pensioen'!$B$29,'5. Verlof &amp; Grootboek'!$B$16,'5. Verlof &amp; Grootboek'!$B$17,'5. Verlof &amp; Grootboek'!$B$18,'6. Akkoord'!$B$8,'6. Akkoord'!$B$9,'6. Akkoord'!$B$11,'6. Akkoord'!$B$12,'6. Akkoord'!$B$15,'6. Akkoord'!$B$16)/36,"0%"),"0%")</f>
         <v/>
       </c>
     </row>
-    <row r="24" ht="22" customHeight="1">
-      <c r="A24" s="5" t="inlineStr">
+    <row r="24" ht="24" customHeight="1">
+      <c r="A24" s="6" t="inlineStr">
         <is>
           <t>Opmerkingen</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="12" t="n"/>
+      <c r="A25" s="13" t="n"/>
     </row>
     <row r="26"/>
     <row r="27"/>
@@ -1068,8 +1291,9 @@
     </dataValidation>
   </dataValidations>
   <printOptions horizontalCentered="1"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
@@ -1093,193 +1317,379 @@
     <col width="28" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
+    <row r="1" ht="55" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>1. Bedrijf &amp; Contact</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="5" t="inlineStr">
+    <row r="2" ht="4" customHeight="1">
+      <c r="A2" s="2" t="n"/>
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+    </row>
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="6" t="inlineStr">
         <is>
           <t>Bedrijfsgegevens</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="13" t="inlineStr">
-        <is>
-          <t>Bedrijfsnaam *</t>
-        </is>
-      </c>
-      <c r="B4" s="7" t="n"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="13" t="inlineStr">
-        <is>
-          <t>Straat + huisnummer *</t>
-        </is>
-      </c>
-      <c r="B5" s="7" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="13" t="inlineStr">
-        <is>
-          <t>Postcode *</t>
-        </is>
-      </c>
-      <c r="B6" s="7" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="13" t="inlineStr">
-        <is>
-          <t>Plaats *</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr">
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="00203040"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Bedrijfsnaam</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="00E01030"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve">  *</t>
+          </r>
+        </is>
+      </c>
+      <c r="B4" s="8" t="n"/>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="00203040"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Straat + huisnummer</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="00E01030"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve">  *</t>
+          </r>
+        </is>
+      </c>
+      <c r="B5" s="8" t="n"/>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="00203040"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Postcode</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="00E01030"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve">  *</t>
+          </r>
+        </is>
+      </c>
+      <c r="B6" s="8" t="n"/>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="00203040"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Plaats</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="00E01030"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve">  *</t>
+          </r>
+        </is>
+      </c>
+      <c r="B7" s="8" t="n"/>
+    </row>
+    <row r="8" ht="18" customHeight="1">
+      <c r="A8" s="7" t="inlineStr">
         <is>
           <t>KvK-nummer</t>
         </is>
       </c>
-      <c r="B8" s="7" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="6" t="inlineStr">
+      <c r="B8" s="8" t="n"/>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
         <is>
           <t>Loonheffingsnummer</t>
         </is>
       </c>
-      <c r="B9" s="7" t="n"/>
-    </row>
-    <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="5" t="inlineStr">
+      <c r="B9" s="8" t="n"/>
+    </row>
+    <row r="11" ht="24" customHeight="1">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t>Contactpersoon HR / salarisadministratie</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="13" t="inlineStr">
-        <is>
-          <t>Naam *</t>
-        </is>
-      </c>
-      <c r="B12" s="7" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="6" t="inlineStr">
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="00203040"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Naam</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="00E01030"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve">  *</t>
+          </r>
+        </is>
+      </c>
+      <c r="B12" s="8" t="n"/>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="7" t="inlineStr">
         <is>
           <t>Functie</t>
         </is>
       </c>
-      <c r="B13" s="7" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="13" t="inlineStr">
-        <is>
-          <t>Telefoon *</t>
-        </is>
-      </c>
-      <c r="B14" s="7" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="13" t="inlineStr">
-        <is>
-          <t>E-mail *</t>
-        </is>
-      </c>
-      <c r="B15" s="7" t="n"/>
-    </row>
-    <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="5" t="inlineStr">
+      <c r="B13" s="8" t="n"/>
+    </row>
+    <row r="14" ht="18" customHeight="1">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="00203040"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Telefoon</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="00E01030"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve">  *</t>
+          </r>
+        </is>
+      </c>
+      <c r="B14" s="8" t="n"/>
+    </row>
+    <row r="15" ht="18" customHeight="1">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="00203040"/>
+              <sz val="11"/>
+            </rPr>
+            <t>E-mail</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="00E01030"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve">  *</t>
+          </r>
+        </is>
+      </c>
+      <c r="B15" s="8" t="n"/>
+    </row>
+    <row r="17" ht="24" customHeight="1">
+      <c r="A17" s="6" t="inlineStr">
         <is>
           <t>Contactpersoon Finance / boekhouding</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="13" t="inlineStr">
-        <is>
-          <t>Naam *</t>
-        </is>
-      </c>
-      <c r="B18" s="7" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="6" t="inlineStr">
+    <row r="18" ht="18" customHeight="1">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="00203040"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Naam</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="00E01030"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve">  *</t>
+          </r>
+        </is>
+      </c>
+      <c r="B18" s="8" t="n"/>
+    </row>
+    <row r="19" ht="18" customHeight="1">
+      <c r="A19" s="7" t="inlineStr">
         <is>
           <t>Functie</t>
         </is>
       </c>
-      <c r="B19" s="7" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="13" t="inlineStr">
-        <is>
-          <t>Telefoon *</t>
-        </is>
-      </c>
-      <c r="B20" s="7" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="13" t="inlineStr">
-        <is>
-          <t>E-mail *</t>
-        </is>
-      </c>
-      <c r="B21" s="7" t="n"/>
-    </row>
-    <row r="23" ht="22" customHeight="1">
-      <c r="A23" s="5" t="inlineStr">
+      <c r="B19" s="8" t="n"/>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="00203040"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Telefoon</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="00E01030"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve">  *</t>
+          </r>
+        </is>
+      </c>
+      <c r="B20" s="8" t="n"/>
+    </row>
+    <row r="21" ht="18" customHeight="1">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="00203040"/>
+              <sz val="11"/>
+            </rPr>
+            <t>E-mail</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="00E01030"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve">  *</t>
+          </r>
+        </is>
+      </c>
+      <c r="B21" s="8" t="n"/>
+    </row>
+    <row r="23" ht="24" customHeight="1">
+      <c r="A23" s="6" t="inlineStr">
         <is>
           <t>Bankgegevens (voor SEPA-betaalbestand nettolonen)</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="13" t="inlineStr">
-        <is>
-          <t>IBAN-rekeningnummer *</t>
-        </is>
-      </c>
-      <c r="B24" s="7" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="6" t="inlineStr">
+    <row r="24" ht="18" customHeight="1">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="00203040"/>
+              <sz val="11"/>
+            </rPr>
+            <t>IBAN-rekeningnummer</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="00E01030"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve">  *</t>
+          </r>
+        </is>
+      </c>
+      <c r="B24" s="8" t="n"/>
+    </row>
+    <row r="25" ht="18" customHeight="1">
+      <c r="A25" s="7" t="inlineStr">
         <is>
           <t>Naam bank</t>
         </is>
       </c>
-      <c r="B25" s="7" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="6" t="inlineStr">
+      <c r="B25" s="8" t="n"/>
+    </row>
+    <row r="26" ht="18" customHeight="1">
+      <c r="A26" s="7" t="inlineStr">
         <is>
           <t>BIC / SWIFT-code</t>
         </is>
       </c>
-      <c r="B26" s="7" t="n"/>
+      <c r="B26" s="8" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="4" t="inlineStr">
+      <c r="A28" s="5" t="inlineStr">
         <is>
           <t>* = verplicht veld. Niet-verplichte velden mogen leeg blijven.</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="22" customHeight="1">
-      <c r="A30" s="5" t="inlineStr">
+    <row r="30" ht="24" customHeight="1">
+      <c r="A30" s="6" t="inlineStr">
         <is>
           <t>Opmerkingen</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="12" t="n"/>
+      <c r="A31" s="13" t="n"/>
     </row>
     <row r="32"/>
     <row r="33"/>
@@ -1296,8 +1706,9 @@
     <mergeCell ref="A17:H17"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
@@ -1321,47 +1732,89 @@
     <col width="28" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
+    <row r="1" ht="55" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>2. Payroll basis</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="5" t="inlineStr">
+    <row r="2" ht="4" customHeight="1">
+      <c r="A2" s="2" t="n"/>
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+    </row>
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="6" t="inlineStr">
         <is>
           <t>CAO (Collectieve arbeidsovereenkomst)</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="13" t="inlineStr">
-        <is>
-          <t>Is een CAO van toepassing? *</t>
-        </is>
-      </c>
-      <c r="B4" s="7" t="n"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="6" t="inlineStr">
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="00203040"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Is een CAO van toepassing?</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="00E01030"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve">  *</t>
+          </r>
+        </is>
+      </c>
+      <c r="B4" s="8" t="n"/>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>Zo ja, welke CAO?</t>
         </is>
       </c>
-      <c r="B5" s="7" t="n"/>
-    </row>
-    <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="B5" s="8" t="n"/>
+    </row>
+    <row r="7" ht="24" customHeight="1">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>Werktijden (standaard fulltime)</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="13" t="inlineStr">
-        <is>
-          <t>Uren per week *</t>
+    <row r="8" ht="18" customHeight="1">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="00203040"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Uren per week</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="00E01030"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve">  *</t>
+          </r>
         </is>
       </c>
       <c r="B8" s="14" t="n">
@@ -1393,39 +1846,55 @@
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="6" t="inlineStr">
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
         <is>
           <t>Uren per dag (maandag - vrijdag)</t>
         </is>
       </c>
-      <c r="C9" s="8" t="n">
+      <c r="C9" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="D9" s="8" t="n">
+      <c r="D9" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="E9" s="8" t="n">
+      <c r="E9" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="F9" s="8" t="n">
+      <c r="F9" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="G9" s="8" t="n">
+      <c r="G9" s="9" t="n">
         <v>8</v>
       </c>
     </row>
-    <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="5" t="inlineStr">
+    <row r="11" ht="24" customHeight="1">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t>Salarisperiode</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="13" t="inlineStr">
-        <is>
-          <t>Salarisperiode *</t>
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="00203040"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Salarisperiode</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="00E01030"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve">  *</t>
+          </r>
         </is>
       </c>
       <c r="B12" s="14" t="inlineStr">
@@ -1434,17 +1903,33 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="5" t="inlineStr">
+    <row r="14" ht="24" customHeight="1">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t>Salarisstrook</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="13" t="inlineStr">
-        <is>
-          <t>Taal salarisstrook *</t>
+    <row r="15" ht="18" customHeight="1">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="00203040"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Taal salarisstrook</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="00E01030"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve">  *</t>
+          </r>
         </is>
       </c>
       <c r="B15" s="14" t="inlineStr">
@@ -1453,18 +1938,50 @@
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="13" t="inlineStr">
-        <is>
-          <t>Logo van uw bedrijf op salarisstrook? *</t>
-        </is>
-      </c>
-      <c r="B16" s="7" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="13" t="inlineStr">
-        <is>
-          <t>Strook zichtbaar voor medewerker *</t>
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="00203040"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Logo van uw bedrijf op salarisstrook?</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="00E01030"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve">  *</t>
+          </r>
+        </is>
+      </c>
+      <c r="B16" s="8" t="n"/>
+    </row>
+    <row r="17" ht="18" customHeight="1">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="00203040"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Strook zichtbaar voor medewerker</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="00E01030"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve">  *</t>
+          </r>
         </is>
       </c>
       <c r="B17" s="14" t="inlineStr">
@@ -1473,25 +1990,41 @@
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="6" t="inlineStr">
+    <row r="18" ht="18" customHeight="1">
+      <c r="A18" s="7" t="inlineStr">
         <is>
           <t>Aantal dagen na betaaldatum</t>
         </is>
       </c>
-      <c r="B18" s="7" t="n"/>
-    </row>
-    <row r="20" ht="22" customHeight="1">
-      <c r="A20" s="5" t="inlineStr">
+      <c r="B18" s="8" t="n"/>
+    </row>
+    <row r="20" ht="24" customHeight="1">
+      <c r="A20" s="6" t="inlineStr">
         <is>
           <t>30%-regeling (voor buitenlandse kenniswerkers)</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="13" t="inlineStr">
-        <is>
-          <t>30%-regeling van toepassing? *</t>
+    <row r="21" ht="18" customHeight="1">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="00203040"/>
+              <sz val="11"/>
+            </rPr>
+            <t>30%-regeling van toepassing?</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="00E01030"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve">  *</t>
+          </r>
         </is>
       </c>
       <c r="B21" s="14" t="inlineStr">
@@ -1500,25 +2033,41 @@
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="6" t="inlineStr">
+    <row r="22" ht="18" customHeight="1">
+      <c r="A22" s="7" t="inlineStr">
         <is>
           <t>Aantal medewerkers met 30%-regeling</t>
         </is>
       </c>
-      <c r="B22" s="7" t="n"/>
-    </row>
-    <row r="24" ht="22" customHeight="1">
-      <c r="A24" s="5" t="inlineStr">
+      <c r="B22" s="8" t="n"/>
+    </row>
+    <row r="24" ht="24" customHeight="1">
+      <c r="A24" s="6" t="inlineStr">
         <is>
           <t>Overige werknemerstypen</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="13" t="inlineStr">
-        <is>
-          <t>Stagiaires in dienst? *</t>
+    <row r="25" ht="18" customHeight="1">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="00203040"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Stagiaires in dienst?</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="00E01030"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve">  *</t>
+          </r>
         </is>
       </c>
       <c r="B25" s="14" t="inlineStr">
@@ -1527,10 +2076,26 @@
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="13" t="inlineStr">
-        <is>
-          <t>Oproepkrachten in dienst? *</t>
+    <row r="26" ht="18" customHeight="1">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="00203040"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Oproepkrachten in dienst?</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="00E01030"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve">  *</t>
+          </r>
         </is>
       </c>
       <c r="B26" s="14" t="inlineStr">
@@ -1539,15 +2104,15 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="22" customHeight="1">
-      <c r="A28" s="5" t="inlineStr">
+    <row r="28" ht="24" customHeight="1">
+      <c r="A28" s="6" t="inlineStr">
         <is>
           <t>Opmerkingen</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="12" t="n"/>
+      <c r="A29" s="13" t="n"/>
     </row>
     <row r="30"/>
     <row r="31"/>
@@ -1586,8 +2151,9 @@
     </dataValidation>
   </dataValidations>
   <printOptions horizontalCentered="1"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
@@ -1611,56 +2177,130 @@
     <col width="28" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
+    <row r="1" ht="55" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>3. Loonheffing</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="5" t="inlineStr">
+    <row r="2" ht="4" customHeight="1">
+      <c r="A2" s="2" t="n"/>
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+    </row>
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="6" t="inlineStr">
         <is>
           <t>Gegevens aangifte loonheffingen</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="13" t="inlineStr">
-        <is>
-          <t>Loonheffingsnummer *</t>
-        </is>
-      </c>
-      <c r="B4" s="7" t="n"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="13" t="inlineStr">
-        <is>
-          <t>Sector (sectorindeling Belastingdienst) *</t>
-        </is>
-      </c>
-      <c r="B5" s="7" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="13" t="inlineStr">
-        <is>
-          <t>Indeling werkgever *</t>
-        </is>
-      </c>
-      <c r="B6" s="7" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="6" t="inlineStr">
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="00203040"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Loonheffingsnummer</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="00E01030"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve">  *</t>
+          </r>
+        </is>
+      </c>
+      <c r="B4" s="8" t="n"/>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="00203040"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Sector (sectorindeling Belastingdienst)</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="00E01030"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve">  *</t>
+          </r>
+        </is>
+      </c>
+      <c r="B5" s="8" t="n"/>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="00203040"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Indeling werkgever</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="00E01030"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve">  *</t>
+          </r>
+        </is>
+      </c>
+      <c r="B6" s="8" t="n"/>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>CBS CAO-code</t>
         </is>
       </c>
-      <c r="B7" s="7" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="13" t="inlineStr">
-        <is>
-          <t>WBSO-subsidie van toepassing? *</t>
+      <c r="B7" s="8" t="n"/>
+    </row>
+    <row r="8" ht="18" customHeight="1">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="00203040"/>
+              <sz val="11"/>
+            </rPr>
+            <t>WBSO-subsidie van toepassing?</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="00E01030"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve">  *</t>
+          </r>
         </is>
       </c>
       <c r="B8" s="14" t="inlineStr">
@@ -1669,8 +2309,8 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="5" t="inlineStr">
+    <row r="10" ht="24" customHeight="1">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>WHK-premie (gedifferentieerde premie Werkhervattingskas)</t>
         </is>
@@ -1688,15 +2328,15 @@
     <row r="12"/>
     <row r="13"/>
     <row r="14"/>
-    <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="5" t="inlineStr">
+    <row r="16" ht="24" customHeight="1">
+      <c r="A16" s="6" t="inlineStr">
         <is>
           <t>Opmerkingen</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="12" t="n"/>
+      <c r="A17" s="13" t="n"/>
     </row>
     <row r="18"/>
     <row r="19"/>
@@ -1723,8 +2363,9 @@
     </dataValidation>
   </dataValidations>
   <printOptions horizontalCentered="1"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
@@ -1748,22 +2389,32 @@
     <col width="28" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
+    <row r="1" ht="55" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>4. Reserveringen &amp; Pensioen</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="5" t="inlineStr">
+    <row r="2" ht="4" customHeight="1">
+      <c r="A2" s="2" t="n"/>
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+    </row>
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="6" t="inlineStr">
         <is>
           <t>Vakantiegeld</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="6" t="inlineStr">
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="7" t="inlineStr">
         <is>
           <t>Uitbetalingspercentage</t>
         </is>
@@ -1774,8 +2425,8 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="6" t="inlineStr">
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>Referentieperiode van</t>
         </is>
@@ -1786,8 +2437,8 @@
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="6" t="inlineStr">
+    <row r="6" ht="18" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>Referentieperiode tot en met</t>
         </is>
@@ -1798,8 +2449,8 @@
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="6" t="inlineStr">
+    <row r="7" ht="18" customHeight="1">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>Uitbetaalmaand</t>
         </is>
@@ -1810,17 +2461,33 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="5" t="inlineStr">
+    <row r="9" ht="24" customHeight="1">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>13e maand</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="13" t="inlineStr">
-        <is>
-          <t>13e maand van toepassing? *</t>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="00203040"/>
+              <sz val="11"/>
+            </rPr>
+            <t>13e maand van toepassing?</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="00E01030"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve">  *</t>
+          </r>
         </is>
       </c>
       <c r="B10" s="14" t="inlineStr">
@@ -1829,28 +2496,44 @@
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="6" t="inlineStr">
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="7" t="inlineStr">
         <is>
           <t>Uitbetaalmaand 13e maand</t>
         </is>
       </c>
-      <c r="B11" s="7" t="n"/>
-    </row>
-    <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="5" t="inlineStr">
+      <c r="B11" s="8" t="n"/>
+    </row>
+    <row r="13" ht="24" customHeight="1">
+      <c r="A13" s="6" t="inlineStr">
         <is>
           <t>Pensioen</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="13" t="inlineStr">
-        <is>
-          <t>Aangesloten bij bedrijfstakpensioenfonds (BPF)? *</t>
-        </is>
-      </c>
-      <c r="B14" s="7" t="n"/>
+    <row r="14" ht="18" customHeight="1">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="00203040"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Aangesloten bij bedrijfstakpensioenfonds (BPF)?</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="00E01030"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve">  *</t>
+          </r>
+        </is>
+      </c>
+      <c r="B14" s="8" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="17" t="inlineStr">
@@ -1859,21 +2542,21 @@
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="6" t="inlineStr">
+    <row r="17" ht="18" customHeight="1">
+      <c r="A17" s="7" t="inlineStr">
         <is>
           <t>Naam bedrijfstakpensioenfonds</t>
         </is>
       </c>
-      <c r="B17" s="7" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="6" t="inlineStr">
+      <c r="B17" s="8" t="n"/>
+    </row>
+    <row r="18" ht="18" customHeight="1">
+      <c r="A18" s="7" t="inlineStr">
         <is>
           <t>Aansluitingsnummer bij het fonds</t>
         </is>
       </c>
-      <c r="B18" s="7" t="n"/>
+      <c r="B18" s="8" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="17" t="inlineStr">
@@ -1882,40 +2565,40 @@
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="6" t="inlineStr">
+    <row r="21" ht="18" customHeight="1">
+      <c r="A21" s="7" t="inlineStr">
         <is>
           <t>Premie werknemer (%)</t>
         </is>
       </c>
-      <c r="B21" s="7" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="6" t="inlineStr">
+      <c r="B21" s="8" t="n"/>
+    </row>
+    <row r="22" ht="18" customHeight="1">
+      <c r="A22" s="7" t="inlineStr">
         <is>
           <t>Premie werkgever (%)</t>
         </is>
       </c>
-      <c r="B22" s="7" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="6" t="inlineStr">
+      <c r="B22" s="8" t="n"/>
+    </row>
+    <row r="23" ht="18" customHeight="1">
+      <c r="A23" s="7" t="inlineStr">
         <is>
           <t>Franchise (EUR per jaar)</t>
         </is>
       </c>
-      <c r="B23" s="7" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="6" t="inlineStr">
+      <c r="B23" s="8" t="n"/>
+    </row>
+    <row r="24" ht="18" customHeight="1">
+      <c r="A24" s="7" t="inlineStr">
         <is>
           <t>Maximum pensioengevend jaarloon (EUR)</t>
         </is>
       </c>
-      <c r="B24" s="7" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="6" t="inlineStr">
+      <c r="B24" s="8" t="n"/>
+    </row>
+    <row r="25" ht="18" customHeight="1">
+      <c r="A25" s="7" t="inlineStr">
         <is>
           <t>Minimum leeftijd voor pensioenopbouw</t>
         </is>
@@ -1924,8 +2607,8 @@
         <v>21</v>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="6" t="inlineStr">
+    <row r="26" ht="18" customHeight="1">
+      <c r="A26" s="7" t="inlineStr">
         <is>
           <t>Maximum leeftijd voor pensioenopbouw</t>
         </is>
@@ -1936,17 +2619,33 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="22" customHeight="1">
-      <c r="A28" s="5" t="inlineStr">
+    <row r="28" ht="24" customHeight="1">
+      <c r="A28" s="6" t="inlineStr">
         <is>
           <t>Aanvullende regelingen</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="13" t="inlineStr">
-        <is>
-          <t>Heeft u aanvullende regelingen? *</t>
+    <row r="29" ht="18" customHeight="1">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="00203040"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Heeft u aanvullende regelingen?</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="00E01030"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve">  *</t>
+          </r>
         </is>
       </c>
       <c r="B29" s="14" t="inlineStr">
@@ -1955,15 +2654,15 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="22" customHeight="1">
-      <c r="A31" s="5" t="inlineStr">
+    <row r="31" ht="24" customHeight="1">
+      <c r="A31" s="6" t="inlineStr">
         <is>
           <t>Geavanceerd (optioneel) - Individueel Keuzebudget (IKB)</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="6" t="inlineStr">
+    <row r="32" ht="18" customHeight="1">
+      <c r="A32" s="7" t="inlineStr">
         <is>
           <t>IKB-toggle</t>
         </is>
@@ -1974,47 +2673,47 @@
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="6" t="inlineStr">
+    <row r="33" ht="18" customHeight="1">
+      <c r="A33" s="7" t="inlineStr">
         <is>
           <t>IKB-percentage</t>
         </is>
       </c>
       <c r="B33" s="14" t="n"/>
     </row>
-    <row r="34">
-      <c r="A34" s="6" t="inlineStr">
+    <row r="34" ht="18" customHeight="1">
+      <c r="A34" s="7" t="inlineStr">
         <is>
           <t>IKB-referentieperiode van</t>
         </is>
       </c>
       <c r="B34" s="14" t="n"/>
     </row>
-    <row r="35">
-      <c r="A35" s="6" t="inlineStr">
+    <row r="35" ht="18" customHeight="1">
+      <c r="A35" s="7" t="inlineStr">
         <is>
           <t>IKB-referentieperiode tot en met</t>
         </is>
       </c>
       <c r="B35" s="14" t="n"/>
     </row>
-    <row r="36">
-      <c r="A36" s="6" t="inlineStr">
+    <row r="36" ht="18" customHeight="1">
+      <c r="A36" s="7" t="inlineStr">
         <is>
           <t>IKB-uitbetaalmaand</t>
         </is>
       </c>
       <c r="B36" s="14" t="n"/>
     </row>
-    <row r="38" ht="22" customHeight="1">
-      <c r="A38" s="5" t="inlineStr">
+    <row r="38" ht="24" customHeight="1">
+      <c r="A38" s="6" t="inlineStr">
         <is>
           <t>Opmerkingen</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="12" t="n"/>
+      <c r="A39" s="13" t="n"/>
     </row>
     <row r="40"/>
     <row r="41"/>
@@ -2043,8 +2742,9 @@
     </dataValidation>
   </dataValidations>
   <printOptions horizontalCentered="1"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
@@ -2068,15 +2768,25 @@
     <col width="28" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
+    <row r="1" ht="55" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>5. Verlof &amp; Grootboek</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="5" t="inlineStr">
+    <row r="2" ht="4" customHeight="1">
+      <c r="A2" s="2" t="n"/>
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+    </row>
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="6" t="inlineStr">
         <is>
           <t>Wettelijke verlofregelingen (WAZO)</t>
         </is>
@@ -2110,15 +2820,15 @@
           <t>Geboorteverlof (1 week)</t>
         </is>
       </c>
-      <c r="B5" s="8" t="n">
+      <c r="B5" s="9" t="n">
         <v>100</v>
       </c>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="C5" s="9" t="inlineStr">
         <is>
           <t>Ja</t>
         </is>
       </c>
-      <c r="D5" s="8" t="inlineStr">
+      <c r="D5" s="9" t="inlineStr">
         <is>
           <t>Ja</t>
         </is>
@@ -2130,15 +2840,15 @@
           <t>Aanvullend geboorteverlof (5 weken)</t>
         </is>
       </c>
-      <c r="B6" s="8" t="n">
+      <c r="B6" s="9" t="n">
         <v>70</v>
       </c>
-      <c r="C6" s="8" t="inlineStr">
+      <c r="C6" s="9" t="inlineStr">
         <is>
           <t>Ja</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="D6" s="9" t="inlineStr">
         <is>
           <t>Nee</t>
         </is>
@@ -2150,15 +2860,15 @@
           <t>Betaald ouderschapsverlof (9 weken)</t>
         </is>
       </c>
-      <c r="B7" s="8" t="n">
+      <c r="B7" s="9" t="n">
         <v>70</v>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="C7" s="9" t="inlineStr">
         <is>
           <t>Ja</t>
         </is>
       </c>
-      <c r="D7" s="8" t="inlineStr">
+      <c r="D7" s="9" t="inlineStr">
         <is>
           <t>Nee</t>
         </is>
@@ -2170,15 +2880,15 @@
           <t>Onbetaald ouderschapsverlof</t>
         </is>
       </c>
-      <c r="B8" s="8" t="n">
+      <c r="B8" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="C8" s="8" t="inlineStr">
+      <c r="C8" s="9" t="inlineStr">
         <is>
           <t>Nee</t>
         </is>
       </c>
-      <c r="D8" s="8" t="inlineStr">
+      <c r="D8" s="9" t="inlineStr">
         <is>
           <t>Nee</t>
         </is>
@@ -2190,15 +2900,15 @@
           <t>Kortdurend zorgverlof</t>
         </is>
       </c>
-      <c r="B9" s="8" t="n">
+      <c r="B9" s="9" t="n">
         <v>70</v>
       </c>
-      <c r="C9" s="8" t="inlineStr">
+      <c r="C9" s="9" t="inlineStr">
         <is>
           <t>Ja</t>
         </is>
       </c>
-      <c r="D9" s="8" t="inlineStr">
+      <c r="D9" s="9" t="inlineStr">
         <is>
           <t>Ja</t>
         </is>
@@ -2210,15 +2920,15 @@
           <t>Langdurig zorgverlof</t>
         </is>
       </c>
-      <c r="B10" s="8" t="n">
+      <c r="B10" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="C10" s="8" t="inlineStr">
+      <c r="C10" s="9" t="inlineStr">
         <is>
           <t>Nee</t>
         </is>
       </c>
-      <c r="D10" s="8" t="inlineStr">
+      <c r="D10" s="9" t="inlineStr">
         <is>
           <t>Nee</t>
         </is>
@@ -2230,54 +2940,102 @@
           <t>Onbetaald verlof (algemeen)</t>
         </is>
       </c>
-      <c r="B11" s="8" t="n">
+      <c r="B11" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="C11" s="8" t="inlineStr">
+      <c r="C11" s="9" t="inlineStr">
         <is>
           <t>Nee</t>
         </is>
       </c>
-      <c r="D11" s="8" t="inlineStr">
+      <c r="D11" s="9" t="inlineStr">
         <is>
           <t>Nee</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t>Defaults = wettelijk minimum. Overschrijf indien uw CAO gunstigere voorwaarden biedt.</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="5" t="inlineStr">
+    <row r="15" ht="24" customHeight="1">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t>Grootboek-export (journaalpost)</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="13" t="inlineStr">
-        <is>
-          <t>Financieel systeem *</t>
-        </is>
-      </c>
-      <c r="B16" s="7" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="13" t="inlineStr">
-        <is>
-          <t>Bestandsformaat export *</t>
-        </is>
-      </c>
-      <c r="B17" s="7" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="13" t="inlineStr">
-        <is>
-          <t>Journaalpost per kostenplaats splitsen? *</t>
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="00203040"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Financieel systeem</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="00E01030"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve">  *</t>
+          </r>
+        </is>
+      </c>
+      <c r="B16" s="8" t="n"/>
+    </row>
+    <row r="17" ht="18" customHeight="1">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="00203040"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Bestandsformaat export</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="00E01030"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve">  *</t>
+          </r>
+        </is>
+      </c>
+      <c r="B17" s="8" t="n"/>
+    </row>
+    <row r="18" ht="18" customHeight="1">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="00203040"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Journaalpost per kostenplaats splitsen?</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="00E01030"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve">  *</t>
+          </r>
         </is>
       </c>
       <c r="B18" s="14" t="inlineStr">
@@ -2295,15 +3053,15 @@
     </row>
     <row r="21"/>
     <row r="22"/>
-    <row r="24" ht="22" customHeight="1">
-      <c r="A24" s="5" t="inlineStr">
+    <row r="24" ht="24" customHeight="1">
+      <c r="A24" s="6" t="inlineStr">
         <is>
           <t>Opmerkingen</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="12" t="n"/>
+      <c r="A25" s="13" t="n"/>
     </row>
     <row r="26"/>
     <row r="27"/>
@@ -2330,8 +3088,9 @@
     </dataValidation>
   </dataValidations>
   <printOptions horizontalCentered="1"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
@@ -2355,12 +3114,22 @@
     <col width="28" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
+    <row r="1" ht="55" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>6. Akkoord</t>
         </is>
       </c>
+    </row>
+    <row r="2" ht="4" customHeight="1">
+      <c r="A2" s="2" t="n"/>
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="20" t="inlineStr">
@@ -2371,85 +3140,181 @@
     </row>
     <row r="4"/>
     <row r="5"/>
-    <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
+    <row r="7" ht="24" customHeight="1">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>Ondertekening</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="13" t="inlineStr">
-        <is>
-          <t>Naam klant / bedrijf *</t>
-        </is>
-      </c>
-      <c r="B8" s="7" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="13" t="inlineStr">
-        <is>
-          <t>Naam ondertekenaar (contactpersoon) *</t>
-        </is>
-      </c>
-      <c r="B9" s="7" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="inlineStr">
+    <row r="8" ht="18" customHeight="1">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="00203040"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Naam klant / bedrijf</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="00E01030"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve">  *</t>
+          </r>
+        </is>
+      </c>
+      <c r="B8" s="8" t="n"/>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="00203040"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Naam ondertekenaar (contactpersoon)</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="00E01030"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve">  *</t>
+          </r>
+        </is>
+      </c>
+      <c r="B9" s="8" t="n"/>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="7" t="inlineStr">
         <is>
           <t>Functie ondertekenaar</t>
         </is>
       </c>
-      <c r="B10" s="7" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="13" t="inlineStr">
-        <is>
-          <t>Datum *</t>
-        </is>
-      </c>
-      <c r="B11" s="7" t="n"/>
+      <c r="B10" s="8" t="n"/>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="00203040"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Datum</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="00E01030"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve">  *</t>
+          </r>
+        </is>
+      </c>
+      <c r="B11" s="8" t="n"/>
     </row>
     <row r="12" ht="60" customHeight="1">
-      <c r="A12" s="13" t="inlineStr">
-        <is>
-          <t>Handtekening *</t>
-        </is>
-      </c>
-      <c r="B12" s="7" t="n"/>
-    </row>
-    <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="5" t="inlineStr">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="00203040"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Handtekening</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="00E01030"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve">  *</t>
+          </r>
+        </is>
+      </c>
+      <c r="B12" s="8" t="n"/>
+    </row>
+    <row r="14" ht="24" customHeight="1">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t>Akkoordverklaringen</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="13" t="inlineStr">
-        <is>
-          <t>Akkoord met de Cobra-setup zoals beschreven in dit document *</t>
-        </is>
-      </c>
-      <c r="B15" s="7" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="13" t="inlineStr">
-        <is>
-          <t>Akkoord met de schaduwverwerking(en) *</t>
-        </is>
-      </c>
-      <c r="B16" s="7" t="n"/>
-    </row>
-    <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="5" t="inlineStr">
+    <row r="15" ht="18" customHeight="1">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="00203040"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Akkoord met de Cobra-setup zoals beschreven in dit document</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="00E01030"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve">  *</t>
+          </r>
+        </is>
+      </c>
+      <c r="B15" s="8" t="n"/>
+    </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="00203040"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Akkoord met de schaduwverwerking(en)</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="00E01030"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve">  *</t>
+          </r>
+        </is>
+      </c>
+      <c r="B16" s="8" t="n"/>
+    </row>
+    <row r="18" ht="24" customHeight="1">
+      <c r="A18" s="6" t="inlineStr">
         <is>
           <t>Opmerkingen</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="12" t="n"/>
+      <c r="A19" s="13" t="n"/>
     </row>
     <row r="20"/>
     <row r="21"/>
@@ -2470,8 +3335,9 @@
     </dataValidation>
   </dataValidations>
   <printOptions horizontalCentered="1"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>

</xml_diff>